<commit_message>
Simplify HOE budget consolidated view as standalone template
Clean template with Consolidated Budget and Definitions sheets only;
no dependency on the existing SharePoint workbook.

Co-authored-by: gayatrirc <gayatri.chandrasekaran@myob.com>
</commit_message>
<xml_diff>
--- a/budget-tools/HOE-Budget-Consolidated-View.xlsx
+++ b/budget-tools/HOE-Budget-Consolidated-View.xlsx
@@ -8,8 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Consolidated Budget" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="How to use" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Column map" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Definitions" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Consolidated Budget'!$A$5:$N$25</definedName>
@@ -153,11 +152,11 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -551,7 +550,7 @@
     <col width="18" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="16" customWidth="1" min="13" max="13"/>
-    <col width="32" customWidth="1" min="14" max="14"/>
+    <col width="28" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -564,14 +563,14 @@
     <row r="2" ht="32" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Roll-up across HOE-maintained budget sheets. Yellow cells = enter/link from source sheets. Green cells = calculated. One row per project / workstream.</t>
+          <t>One row per project / workstream. Yellow = enter values. Green = calculated. Use this as the roll-up across HOE-owned budgets.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Template created: 2026-10-06  |  Currency: AUD  |  Classification: Restricted (financial)</t>
+          <t>Template  |  Currency: AUD  |  Classification: Restricted (financial)  |  Created 2026-10-06</t>
         </is>
       </c>
     </row>
@@ -643,32 +642,16 @@
       </c>
       <c r="N5" s="4" t="inlineStr">
         <is>
-          <t>Notes / Source sheet</t>
+          <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>Example: Project Alpha</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>FY26</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>HOE Name</t>
-        </is>
-      </c>
+      <c r="A6" s="5" t="inlineStr"/>
+      <c r="B6" s="6" t="n"/>
+      <c r="C6" s="6" t="n"/>
       <c r="D6" s="7" t="n"/>
-      <c r="E6" s="6" t="inlineStr">
-        <is>
-          <t>Approver Name</t>
-        </is>
-      </c>
+      <c r="E6" s="6" t="n"/>
       <c r="F6" s="8" t="n"/>
       <c r="G6" s="7" t="n"/>
       <c r="H6" s="7" t="n"/>
@@ -689,34 +672,14 @@
         <f>IF(OR(D6="",I6=""),"",I6-D6)</f>
         <v/>
       </c>
-      <c r="N6" s="5" t="inlineStr">
-        <is>
-          <t>Replace with real project; link figures from HOE sheet</t>
-        </is>
-      </c>
+      <c r="N6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>Example: Project Beta</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>FY26</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>HOE Name</t>
-        </is>
-      </c>
+      <c r="A7" s="5" t="n"/>
+      <c r="B7" s="6" t="n"/>
+      <c r="C7" s="6" t="n"/>
       <c r="D7" s="7" t="n"/>
-      <c r="E7" s="6" t="inlineStr">
-        <is>
-          <t>Approver Name</t>
-        </is>
-      </c>
+      <c r="E7" s="6" t="n"/>
       <c r="F7" s="8" t="n"/>
       <c r="G7" s="7" t="n"/>
       <c r="H7" s="7" t="n"/>
@@ -737,11 +700,7 @@
         <f>IF(OR(D7="",I7=""),"",I7-D7)</f>
         <v/>
       </c>
-      <c r="N7" s="5" t="inlineStr">
-        <is>
-          <t>Delete example rows once live data is entered</t>
-        </is>
-      </c>
+      <c r="N7" s="5" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="n"/>
@@ -1282,7 +1241,7 @@
         <v/>
       </c>
       <c r="L26" s="13">
-        <f>IF(D26=0,"",G26/D26)</f>
+        <f>IF(OR(D26="",D26=0),"",G26/D26)</f>
         <v/>
       </c>
       <c r="M26" s="12">
@@ -1306,7 +1265,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Manual input or cross-sheet link from each HOE budget sheet</t>
+          <t>Enter / paste values</t>
         </is>
       </c>
     </row>
@@ -1318,7 +1277,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Calculated — do not overwrite (Allocated, Remaining, % Spent, Forecast vs Approved)</t>
+          <t>Calculated — do not overwrite</t>
         </is>
       </c>
     </row>
@@ -1330,7 +1289,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Totals across all projects</t>
+          <t>Totals</t>
         </is>
       </c>
     </row>
@@ -1366,241 +1325,197 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="90" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="80" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>How to add this sheet to the existing HOE budget workbook</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="36" customHeight="1">
+          <t>Column definitions</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
       <c r="A3" s="18" t="inlineStr">
         <is>
-          <t>Purpose</t>
-        </is>
-      </c>
-      <c r="B3" s="19" t="inlineStr">
-        <is>
-          <t>Give leadership one consolidated view of where engineering project money is going across HOE-owned sheets.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="36" customHeight="1">
-      <c r="A4" s="18" t="inlineStr">
-        <is>
-          <t>Columns (required)</t>
-        </is>
-      </c>
-      <c r="B4" s="19" t="inlineStr">
-        <is>
-          <t>Total Budget Approved | Approved By | Managed by (HOE) | Spent (Actual) | Unallocated | Forecasted Spend — plus Project, Period, and calculated Remaining / % Spent.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="36" customHeight="1">
-      <c r="A5" s="18" t="inlineStr">
-        <is>
-          <t>Step 1</t>
-        </is>
-      </c>
-      <c r="B5" s="19" t="inlineStr">
-        <is>
-          <t>Open the existing shared Excel (Vivying / HOE budget workbook) in Excel for the web or desktop.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="36" customHeight="1">
-      <c r="A6" s="18" t="inlineStr">
-        <is>
-          <t>Step 2</t>
-        </is>
-      </c>
-      <c r="B6" s="19" t="inlineStr">
-        <is>
-          <t>Right-click any sheet tab → Move or Copy → create a new blank sheet, rename it Consolidated Budget — or copy this entire workbook's Consolidated Budget sheet into that file (right-click tab → Move or Copy → check Create a copy → select the target workbook).</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="36" customHeight="1">
-      <c r="A7" s="18" t="inlineStr">
-        <is>
-          <t>Step 3</t>
-        </is>
-      </c>
-      <c r="B7" s="19" t="inlineStr">
-        <is>
-          <t>For each project row, enter or link: Project name, FY/Period, Managed by (HOE), Total Budget Approved, Approved By, Approval Date, Spent, Unallocated, Forecasted Spend.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="36" customHeight="1">
-      <c r="A8" s="18" t="inlineStr">
-        <is>
-          <t>Step 4</t>
-        </is>
-      </c>
-      <c r="B8" s="19" t="inlineStr">
-        <is>
-          <t>Prefer Excel links to HOE detail sheets, e.g. ='HOE Alpha'!B12, so the rollup stays live. Do not paste stale snapshots if a source sheet already has the figure.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="18" t="inlineStr">
-        <is>
-          <t>Definitions</t>
-        </is>
-      </c>
-      <c r="B9" s="19" t="inlineStr"/>
-    </row>
-    <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="18" t="inlineStr">
+          <t>Column</t>
+        </is>
+      </c>
+      <c r="B3" s="18" t="inlineStr">
+        <is>
+          <t>Meaning</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="19" t="inlineStr">
+        <is>
+          <t>Project / Workstream</t>
+        </is>
+      </c>
+      <c r="B4" s="20" t="inlineStr">
+        <is>
+          <t>Name of the project or workstream being tracked.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="19" t="inlineStr">
+        <is>
+          <t>FY / Period</t>
+        </is>
+      </c>
+      <c r="B5" s="20" t="inlineStr">
+        <is>
+          <t>Financial year or period the approval covers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="19" t="inlineStr">
+        <is>
+          <t>Managed by (HOE)</t>
+        </is>
+      </c>
+      <c r="B6" s="20" t="inlineStr">
+        <is>
+          <t>Head of Engineering accountable for managing spend against the approved amount.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="19" t="inlineStr">
         <is>
           <t>Total Budget Approved</t>
         </is>
       </c>
-      <c r="B10" s="19" t="inlineStr">
+      <c r="B7" s="20" t="inlineStr">
         <is>
           <t>Full amount formally approved for the project/workstream for the period.</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="18" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="19" t="inlineStr">
         <is>
           <t>Approved By</t>
         </is>
       </c>
-      <c r="B11" s="19" t="inlineStr">
-        <is>
-          <t>Person (or forum) that approved the budget.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="18" t="inlineStr">
-        <is>
-          <t>Managed by (HOE)</t>
-        </is>
-      </c>
-      <c r="B12" s="19" t="inlineStr">
-        <is>
-          <t>Head of Engineering accountable for managing spend against the approved amount.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="18" t="inlineStr">
+      <c r="B8" s="20" t="inlineStr">
+        <is>
+          <t>Person or forum that approved the budget.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="19" t="inlineStr">
+        <is>
+          <t>Approval Date</t>
+        </is>
+      </c>
+      <c r="B9" s="20" t="inlineStr">
+        <is>
+          <t>Date the budget was approved.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="19" t="inlineStr">
         <is>
           <t>Spent (Actual)</t>
         </is>
       </c>
-      <c r="B13" s="19" t="inlineStr">
+      <c r="B10" s="20" t="inlineStr">
         <is>
           <t>Amount already incurred / booked against the approved budget to date.</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="36" customHeight="1">
-      <c r="A14" s="18" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="19" t="inlineStr">
         <is>
           <t>Unallocated</t>
         </is>
       </c>
-      <c r="B14" s="19" t="inlineStr">
-        <is>
-          <t>Portion of approved budget not yet assigned to a specific line / vendor / work package.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="36" customHeight="1">
-      <c r="A15" s="18" t="inlineStr">
+      <c r="B11" s="20" t="inlineStr">
+        <is>
+          <t>Portion of approved budget not yet assigned to a line, vendor, or work package.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="19" t="inlineStr">
         <is>
           <t>Forecasted Spend</t>
         </is>
       </c>
-      <c r="B15" s="19" t="inlineStr">
-        <is>
-          <t>Expected total spend to end of period (committed + planned), not only what is spent today.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="18" t="inlineStr">
+      <c r="B12" s="20" t="inlineStr">
+        <is>
+          <t>Expected total spend to end of period (committed + planned).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="19" t="inlineStr">
         <is>
           <t>Allocated (calc)</t>
         </is>
       </c>
-      <c r="B16" s="19" t="inlineStr">
+      <c r="B13" s="20" t="inlineStr">
         <is>
           <t>Approved − Unallocated.</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="18" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="19" t="inlineStr">
         <is>
           <t>Remaining (calc)</t>
         </is>
       </c>
-      <c r="B17" s="19" t="inlineStr">
+      <c r="B14" s="20" t="inlineStr">
         <is>
           <t>Approved − Spent.</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="18" t="inlineStr">
-        <is>
-          <t>% Spent (calc)</t>
-        </is>
-      </c>
-      <c r="B18" s="19" t="inlineStr">
-        <is>
-          <t>Spent ÷ Approved.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="18" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="19" t="inlineStr">
+        <is>
+          <t>% of Approved Spent (calc)</t>
+        </is>
+      </c>
+      <c r="B15" s="20" t="inlineStr">
+        <is>
+          <t>Spent ÷ Approved. Highlights red above 90%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="19" t="inlineStr">
         <is>
           <t>Forecast vs Approved (calc)</t>
         </is>
       </c>
-      <c r="B19" s="19" t="inlineStr">
-        <is>
-          <t>Forecasted Spend − Approved (positive = forecast overspend).</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="36" customHeight="1">
-      <c r="A20" s="18" t="inlineStr">
-        <is>
-          <t>Security</t>
-        </is>
-      </c>
-      <c r="B20" s="19" t="inlineStr">
-        <is>
-          <t>Treat as Restricted financial data: limit sharing to need-to-know, do not put PII beyond names/roles needed for accountability, do not commit live figures to public repos.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="36" customHeight="1">
-      <c r="A21" s="18" t="inlineStr">
-        <is>
-          <t>Limitation</t>
-        </is>
-      </c>
-      <c r="B21" s="19" t="inlineStr">
-        <is>
-          <t>This agent could not write directly to the SharePoint/OneDrive file (personal library of vivying.cheng@myob.com is not reachable from the cloud agent network). Copy this sheet into that workbook, or re-upload the .xlsx here so the sheet can be merged automatically.</t>
+      <c r="B16" s="20" t="inlineStr">
+        <is>
+          <t>Forecasted Spend − Approved. Positive (red) means forecast overspend.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="19" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="B17" s="20" t="inlineStr">
+        <is>
+          <t>Free-text context or link to the HOE detail sheet.</t>
         </is>
       </c>
     </row>
@@ -1610,357 +1525,4 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D17"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
-  <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="55" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Column map — Consolidated Budget</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="20" t="inlineStr">
-        <is>
-          <t>Column</t>
-        </is>
-      </c>
-      <c r="B3" s="20" t="inlineStr">
-        <is>
-          <t>Field</t>
-        </is>
-      </c>
-      <c r="C3" s="20" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="D3" s="20" t="inlineStr">
-        <is>
-          <t>Source</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Project / Workstream</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Input</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Name of project or workstream</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>FY / Period</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Input</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Financial year or period the approval covers</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Managed by (HOE)</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Input</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Accountable Head of Engineering</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Total Budget Approved</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Input</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>From approval record / HOE sheet</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Approved By</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Input</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Approver name or forum</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Approval Date</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Input</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Date of approval</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Spent (Actual)</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Input</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>From HOE sheet / finance actuals</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>H</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Unallocated</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Input</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Approved amount not yet allocated</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Forecasted Spend</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Input</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>From HOE forecast</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>J</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Allocated</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Formula</t>
-        </is>
-      </c>
-      <c r="D13">
-        <f> Approved − Unallocated</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>K</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Remaining (Approved − Spent)</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Formula</t>
-        </is>
-      </c>
-      <c r="D14">
-        <f> Approved − Spent</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>% of Approved Spent</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Formula</t>
-        </is>
-      </c>
-      <c r="D15">
-        <f> Spent ÷ Approved</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Forecast vs Approved</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Formula</t>
-        </is>
-      </c>
-      <c r="D16">
-        <f> Forecasted Spend − Approved</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Notes / Source sheet</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Input</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Link or tab name of the HOE detail sheet</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>